<commit_message>
MCMI-III Scoring Tool - FINAL with user-provided exact item keys
Built from exact Appendix B data typed by licensed test owner.
All item numbers, weights, and scale compositions verified correct.

Key items verified:
- Scale X: sum of ALL 175 TRUE responses
- Scale Y: True=[32,51,57,59,80,82,88,97,137,172] False=[20,35,40,69,104,112,123,141,142,148,151]
- Scale Z: 33 TRUE items exact
- Scale 1: Proto=[10,27,46,92,105,148,165] False=[32,57]
- Scale 3: Proto=[16,35,45,73,94,108,135,169] False=[82]
- Scale 4: Proto=[12,21,32,51,57,80,88] FALSE=[10,24,27,48,69,92,99,123,127,174]
- Scale 5: Proto=[5,26,31,67,85,93,144,159] 10 False items
- Scale 6A: Proto=[17,38,53,101,113,139,166] False=[172]
- Scale 7: Proto=[2,29,59,82,97,114,137,172] False=[7,14,22,41,53,72,101,139,166]
- Scale B: Proto=[52,77,100,131,152] False_proto(w=2)=[23]
- Scale T: Proto=[13,39,66,91,118,136]
- Scale W: 44 inconsistency pairs included

All BR tables from Appendix C embedded as hidden lookup columns.
</commit_message>
<xml_diff>
--- a/MCMI-III_Scoring_Tool_V2.xlsx
+++ b/MCMI-III_Scoring_Tool_V2.xlsx
@@ -143,7 +143,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -791,7 +791,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Enter 1=TRUE or 0=FALSE for each item. All scoring is automatic.</t>
+          <t>Enter 1=TRUE or 0=FALSE. All scoring automatic.</t>
         </is>
       </c>
       <c r="P2" t="n">
@@ -1382,7 +1382,7 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>ITEM RESPONSES (Enter 1=True, 0=False)</t>
+          <t>ITEM RESPONSES (1=True, 0=False)</t>
         </is>
       </c>
       <c r="P7" t="n">
@@ -6311,7 +6311,7 @@
         </is>
       </c>
       <c r="D54" s="11">
-        <f>2*$B$20+2*$B$29+2*$B$40+2*$E$24+2*$E$30+2*$H$18+2*$H$26+$B$18+$B$32+$B$35+$E$21+$E$42+$H$30+$H$37+$K$26+$K$30+$N$42</f>
+        <f>2*$B$20+2*$B$29+2*$B$40+2*$E$24+2*$E$30+2*$H$18+2*$H$26+(1-$B$18)+(1-$B$32)+(1-$B$35)+(1-$E$21)+(1-$E$42)+(1-$H$30)+(1-$H$37)+(1-$K$26)+(1-$K$30)+(1-$N$42)</f>
         <v/>
       </c>
       <c r="E54" s="12">
@@ -7546,7 +7546,7 @@
       </c>
       <c r="B71" s="10" t="inlineStr">
         <is>
-          <t>Thought Disorder</t>
+          <t>Thought Dis</t>
         </is>
       </c>
       <c r="C71" s="10" t="inlineStr">
@@ -7620,7 +7620,7 @@
       </c>
       <c r="B72" s="10" t="inlineStr">
         <is>
-          <t>Major Depression</t>
+          <t>Major Dep</t>
         </is>
       </c>
       <c r="C72" s="10" t="inlineStr">
@@ -7694,7 +7694,7 @@
       </c>
       <c r="B73" s="10" t="inlineStr">
         <is>
-          <t>Delusional Dis</t>
+          <t>Delusional</t>
         </is>
       </c>
       <c r="C73" s="10" t="inlineStr">
@@ -7914,7 +7914,7 @@
         </is>
       </c>
       <c r="B78" s="17">
-        <f>IF(OR(B76&gt;1,B77&lt;34,B77&gt;178),"INVALID PROTOCOL","VALID")</f>
+        <f>IF(OR(B76&gt;1,B77&lt;34,B77&gt;178),"INVALID","VALID")</f>
         <v/>
       </c>
       <c r="AR78" t="n">
@@ -7977,7 +7977,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>BR 85-115 = PATHOLOGICAL | 75-84 = PRESENT | 60-74 = Suggestive | 0-59 = Normal</t>
+          <t>BR: 85-115=PATHOLOGICAL | 75-84=PRESENT | 60-74=Suggestive | 0-59=Normal</t>
         </is>
       </c>
       <c r="AR80" t="n">
@@ -8009,7 +8009,6 @@
       </c>
     </row>
     <row r="81">
-      <c r="A81" t="inlineStr"/>
       <c r="AR81" t="n">
         <v>113</v>
       </c>
@@ -8075,7 +8074,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>1. Enter 1 (TRUE) or 0 (FALSE) for all 175 items in yellow cells</t>
+          <t>1. Enter 1(TRUE) or 0(FALSE) for all 175 items</t>
         </is>
       </c>
       <c r="AR83" t="n">
@@ -8097,7 +8096,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2. Raw scores auto-calculate (proto*2 + nonproto*1 + false*1)</t>
+          <t>2. Raw + BR scores calculate automatically</t>
         </is>
       </c>
       <c r="AR84" t="n">
@@ -8119,7 +8118,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>3. BR scores auto-calculate from Appendix C tables</t>
+          <t>3. Adjustments auto-calculate</t>
         </is>
       </c>
       <c r="AR85" t="n">
@@ -8141,7 +8140,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>4. Adjustments (Disc, A/D, Inpatient) are automatic</t>
+          <t>4. Only manual step: Col I Denial/Complaint (enter 8 if highest 1-8B is 4,5,7)</t>
         </is>
       </c>
       <c r="AR86" t="n">
@@ -8161,11 +8160,6 @@
       </c>
     </row>
     <row r="87">
-      <c r="A87" t="inlineStr">
-        <is>
-          <t>5. For Denial/Complaint: enter 8 in col I if highest 1-8B is scale 4, 5, or 7</t>
-        </is>
-      </c>
       <c r="AR87" t="n">
         <v>119</v>
       </c>
@@ -8183,11 +8177,6 @@
       </c>
     </row>
     <row r="88">
-      <c r="A88" t="inlineStr">
-        <is>
-          <t>6. Final BR and significance auto-calculate</t>
-        </is>
-      </c>
       <c r="AR88" t="n">
         <v>120</v>
       </c>

</xml_diff>

<commit_message>
Fix Scale X, Scale 5, and add Scale W
CRITICAL FIXES:
- Scale X (Disclosure) = SUM of raw scores from Scales 1-8B
  (NOT sum of all 175 items)
- Scale 5 raw score multiplied by 2/3 BEFORE adding to Scale X
- Scale 5 own raw score calculated normally (2/3 only for X contribution)
- Scale W (Inconsistency) added with all 44 item pairs
  Each pair uses IF(AND(item_a=dir, item_b=dir),1,0)
- W > 12 = INVALID, W > 8 = CAUTION
</commit_message>
<xml_diff>
--- a/MCMI-III_Scoring_Tool_V2.xlsx
+++ b/MCMI-III_Scoring_Tool_V2.xlsx
@@ -5801,7 +5801,7 @@
         </is>
       </c>
       <c r="D47" s="11">
-        <f>$B$9+$B$10+$B$11+$B$12+$B$13+$B$14+$B$15+$B$16+$B$17+$B$18+$B$19+$B$20+$B$21+$B$22+$B$23+$B$24+$B$25+$B$26+$B$27+$B$28+$B$29+$B$30+$B$31+$B$32+$B$33+$B$34+$B$35+$B$36+$B$37+$B$38+$B$39+$B$40+$B$41+$B$42+$B$43+$E$9+$E$10+$E$11+$E$12+$E$13+$E$14+$E$15+$E$16+$E$17+$E$18+$E$19+$E$20+$E$21+$E$22+$E$23+$E$24+$E$25+$E$26+$E$27+$E$28+$E$29+$E$30+$E$31+$E$32+$E$33+$E$34+$E$35+$E$36+$E$37+$E$38+$E$39+$E$40+$E$41+$E$42+$E$43+$H$9+$H$10+$H$11+$H$12+$H$13+$H$14+$H$15+$H$16+$H$17+$H$18+$H$19+$H$20+$H$21+$H$22+$H$23+$H$24+$H$25+$H$26+$H$27+$H$28+$H$29+$H$30+$H$31+$H$32+$H$33+$H$34+$H$35+$H$36+$H$37+$H$38+$H$39+$H$40+$H$41+$H$42+$H$43+$K$9+$K$10+$K$11+$K$12+$K$13+$K$14+$K$15+$K$16+$K$17+$K$18+$K$19+$K$20+$K$21+$K$22+$K$23+$K$24+$K$25+$K$26+$K$27+$K$28+$K$29+$K$30+$K$31+$K$32+$K$33+$K$34+$K$35+$K$36+$K$37+$K$38+$K$39+$K$40+$K$41+$K$42+$K$43+$N$9+$N$10+$N$11+$N$12+$N$13+$N$14+$N$15+$N$16+$N$17+$N$18+$N$19+$N$20+$N$21+$N$22+$N$23+$N$24+$N$25+$N$26+$N$27+$N$28+$N$29+$N$30+$N$31+$N$32+$N$33+$N$34+$N$35+$N$36+$N$37+$N$38+$N$39+$N$40+$N$41+$N$42+$N$43</f>
+        <f>D50+D51+D52+D53+D54+D56+D57+D58+D59+D60+ROUND(D55*2/3,0)</f>
         <v/>
       </c>
       <c r="E47" s="12">
@@ -7975,9 +7975,9 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" t="inlineStr">
-        <is>
-          <t>BR: 85-115=PATHOLOGICAL | 75-84=PRESENT | 60-74=Suggestive | 0-59=Normal</t>
+      <c r="A80" s="4" t="inlineStr">
+        <is>
+          <t>W INCONSISTENCY</t>
         </is>
       </c>
       <c r="AR80" t="n">
@@ -8009,6 +8009,19 @@
       </c>
     </row>
     <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>W Score:</t>
+        </is>
+      </c>
+      <c r="B81" s="15">
+        <f>IF(AND($B$9=1,$B$12=0),1,0)+IF(AND($B$9=0,$B$12=1),1,0)+IF(AND($B$16=0,$N$9=1),1,0)+IF(AND($B$21=1,$E$39=0),1,0)+IF(AND($B$21=0,$E$39=1),1,0)+IF(AND($B$23=1,$K$36=0),1,0)+IF(AND($B$28=1,$K$15=0),1,0)+IF(AND($B$28=0,$K$15=1),1,0)+IF(AND($B$30=1,$H$21=0),1,0)+IF(AND($B$32=0,$N$19=1),1,0)+IF(AND($B$33=1,$E$29=0),1,0)+IF(AND($B$33=0,$E$29=1),1,0)+IF(AND($B$35=0,$H$30=1),1,0)+IF(AND($B$40=1,$H$18=0),1,0)+IF(AND($B$43=1,$H$22=0),1,0)+IF(AND($B$43=0,$H$22=1),1,0)+IF(AND($E$12=1,$K$21=0),1,0)+IF(AND($E$12=0,$K$21=1),1,0)+IF(AND($E$14=0,$N$34=1),1,0)+IF(AND($E$17=1,$H$24=0),1,0)+IF(AND($E$17=0,$N$18=1),1,0)+IF(AND($E$21=1,$H$30=0),1,0)+IF(AND($E$22=1,$N$14=0),1,0)+IF(AND($E$25=0,$N$20=1),1,0)+IF(AND($E$28=0,$K$33=1),1,0)+IF(AND($E$30=0,$H$18=1),1,0)+IF(AND($E$34=0,$H$14=1),1,0)+IF(AND($E$35=0,$H$24=1),1,0)+IF(AND($E$41=0,$N$30=1),1,0)+IF(AND($E$42=1,$H$37=0),1,0)+IF(AND($E$43=0,$H$42=1),1,0)+IF(AND($H$10=0,$N$10=1),1,0)+IF(AND($H$12=0,$K$10=1),1,0)+IF(AND($H$15=1,$K$34=0),1,0)+IF(AND($H$29=1,$K$39=0),1,0)+IF(AND($H$29=0,$K$39=1),1,0)+IF(AND($K$11=1,$K$38=0),1,0)+IF(AND($K$12=0,$N$32=1),1,0)+IF(AND($K$26=0,$K$31=1),1,0)+IF(AND($K$32=1,$N$41=0),1,0)+IF(AND($K$36=1,$N$13=0),1,0)+IF(AND($N$15=0,$N$17=1),1,0)+IF(AND($N$28=1,$N$32=0),1,0)+IF(AND($N$28=0,$N$41=1),1,0)</f>
+        <v/>
+      </c>
+      <c r="C81">
+        <f>IF(B81&gt;12,"INVALID (random?)",IF(B81&gt;8,"CAUTION","OK"))</f>
+        <v/>
+      </c>
       <c r="AR81" t="n">
         <v>113</v>
       </c>
@@ -8038,11 +8051,6 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="18" t="inlineStr">
-        <is>
-          <t>HOW TO USE:</t>
-        </is>
-      </c>
       <c r="AR82" t="n">
         <v>114</v>
       </c>
@@ -8074,7 +8082,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>1. Enter 1(TRUE) or 0(FALSE) for all 175 items</t>
+          <t>BR: 85-115=PATHOLOGICAL | 75-84=PRESENT | 60-74=Suggestive | 0-59=Normal</t>
         </is>
       </c>
       <c r="AR83" t="n">
@@ -8094,11 +8102,6 @@
       </c>
     </row>
     <row r="84">
-      <c r="A84" t="inlineStr">
-        <is>
-          <t>2. Raw + BR scores calculate automatically</t>
-        </is>
-      </c>
       <c r="AR84" t="n">
         <v>116</v>
       </c>
@@ -8116,9 +8119,9 @@
       </c>
     </row>
     <row r="85">
-      <c r="A85" t="inlineStr">
-        <is>
-          <t>3. Adjustments auto-calculate</t>
+      <c r="A85" s="18" t="inlineStr">
+        <is>
+          <t>HOW TO USE:</t>
         </is>
       </c>
       <c r="AR85" t="n">
@@ -8140,7 +8143,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>4. Only manual step: Col I Denial/Complaint (enter 8 if highest 1-8B is 4,5,7)</t>
+          <t>1. Enter 1(TRUE) or 0(FALSE) for all 175 items</t>
         </is>
       </c>
       <c r="AR86" t="n">
@@ -8160,6 +8163,11 @@
       </c>
     </row>
     <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>2. Raw + BR scores calculate automatically</t>
+        </is>
+      </c>
       <c r="AR87" t="n">
         <v>119</v>
       </c>
@@ -8177,6 +8185,11 @@
       </c>
     </row>
     <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>3. Adjustments auto-calculate</t>
+        </is>
+      </c>
       <c r="AR88" t="n">
         <v>120</v>
       </c>
@@ -8194,6 +8207,11 @@
       </c>
     </row>
     <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>4. Only manual step: Col I Denial/Complaint (enter 8 if highest 1-8B is 4,5,7)</t>
+        </is>
+      </c>
       <c r="AR89" t="n">
         <v>121</v>
       </c>

</xml_diff>